<commit_message>
fix: layout, data format, actual data
</commit_message>
<xml_diff>
--- a/data_set/data.xlsx
+++ b/data_set/data.xlsx
@@ -5,10 +5,10 @@
   <workbookPr checkCompatibility="1" defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\FMIS\Tech-project\R20-dashboard\New folder\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\FMIS\Tech-project\R20-dashboard\data_set\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4454D99C-C300-4160-9B95-461FAD65AD2B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6435E27B-7BCE-400C-A647-E3AC1D30BBA1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="33">
   <si>
     <t xml:space="preserve">   </t>
   </si>
@@ -138,6 +138,9 @@
   </si>
   <si>
     <t>Q4</t>
+  </si>
+  <si>
+    <t>(-10393900000000)</t>
   </si>
 </sst>
 </file>
@@ -146,7 +149,7 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="2">
     <numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="166" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="164" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
   </numFmts>
   <fonts count="3" x14ac:knownFonts="1">
     <font>
@@ -207,16 +210,16 @@
   </cellStyleXfs>
   <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="166" fontId="2" fillId="2" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="164" fontId="2" fillId="2" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="166" fontId="2" fillId="3" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="164" fontId="2" fillId="3" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="43" fontId="2" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="166" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="49" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
-    <xf numFmtId="166" fontId="0" fillId="3" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
@@ -562,10 +565,10 @@
   <cols>
     <col min="1" max="1" width="4.125" style="7" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="13.25" style="7" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="18" style="7" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="25" style="7" customWidth="1"/>
     <col min="4" max="4" width="23.75" style="7" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="20.625" style="7" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="17.875" style="7" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="21" style="7" customWidth="1"/>
     <col min="7" max="7" width="20.25" style="7" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="21.5" style="7" bestFit="1" customWidth="1"/>
     <col min="9" max="16384" width="9.125" style="7"/>
@@ -664,8 +667,8 @@
       <c r="D4" s="7">
         <v>1016670000000</v>
       </c>
-      <c r="E4" s="7">
-        <v>10393900000000</v>
+      <c r="E4" s="7" t="s">
+        <v>32</v>
       </c>
       <c r="F4" s="7">
         <v>8277340000000</v>
@@ -696,10 +699,10 @@
       </c>
       <c r="E5" s="7">
         <f>SUM(E2:E4)</f>
-        <v>17566900000000</v>
+        <v>7173000000000</v>
       </c>
       <c r="F5" s="7">
-        <f t="shared" si="1"/>
+        <f>SUM(F2:F4)</f>
         <v>37783358000000</v>
       </c>
       <c r="G5" s="7">

</xml_diff>